<commit_message>
Add advanced enterprise Dashboard Excel
</commit_message>
<xml_diff>
--- a/Data_Analyst_Assignment/Spreadsheets/Ticket_Analysis.xlsx
+++ b/Data_Analyst_Assignment/Spreadsheets/Ticket_Analysis.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ticket" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="feedbacks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Analysis Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ticket" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="feedbacks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,16 +27,35 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00366092"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +63,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,91 +455,141 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticket_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>closed_at</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>outlet_id</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>cms_id</t>
-        </is>
-      </c>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticket Resolution Time Analysis</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>isu-sjd-457</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2021-08-19 16:45:43</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2021-08-22 12:33:32</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Outlet ID</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Total Tickets</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Closed Same Day</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Closed Same Hour</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Same Hour %</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>wrqy-juv-978</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>vew-iuvd-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>qer-fal-092</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2021-08-21 11:09:22</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2021-08-21 17:13:45</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="B5" s="2">
+        <f>COUNTIF(ticket!D:D, "wrqy-juv-978")</f>
+        <v/>
+      </c>
+      <c r="C5" s="2">
+        <f>COUNTIFS(ticket!D:D, "wrqy-juv-978", ticket!F:F, "Yes")</f>
+        <v/>
+      </c>
+      <c r="D5" s="2">
+        <f>COUNTIFS(ticket!D:D, "wrqy-juv-978", ticket!G:G, "Yes")</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>IF(B5=0, 0, D5/B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>8woh-k3u-23b</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>qwe-asd-99</t>
-        </is>
+      <c r="B6" s="2">
+        <f>COUNTIF(ticket!D:D, "8woh-k3u-23b")</f>
+        <v/>
+      </c>
+      <c r="C6" s="2">
+        <f>COUNTIFS(ticket!D:D, "8woh-k3u-23b", ticket!F:F, "Yes")</f>
+        <v/>
+      </c>
+      <c r="D6" s="2">
+        <f>COUNTIFS(ticket!D:D, "8woh-k3u-23b", ticket!G:G, "Yes")</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>IF(B6=0, 0, D6/B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>outlet-alpha</t>
+        </is>
+      </c>
+      <c r="B7" s="2">
+        <f>COUNTIF(ticket!D:D, "outlet-alpha")</f>
+        <v/>
+      </c>
+      <c r="C7" s="2">
+        <f>COUNTIFS(ticket!D:D, "outlet-alpha", ticket!F:F, "Yes")</f>
+        <v/>
+      </c>
+      <c r="D7" s="2">
+        <f>COUNTIFS(ticket!D:D, "outlet-alpha", ticket!G:G, "Yes")</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>IF(B7=0, 0, D7/B7)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -509,66 +600,523 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="39" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>ticket_id</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>closed_at</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>outlet_id</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>cms_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>same_day_flag</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>same_hour_flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>isu-sjd-457</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-19 16:45:43</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-22 12:33:32</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>wrqy-juv-978</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>vew-iuvd-12</t>
+        </is>
+      </c>
+      <c r="F2" s="2">
+        <f>IF(INT(B2)=INT(C2), "Yes", "No")</f>
+        <v/>
+      </c>
+      <c r="G2" s="2">
+        <f>IF(AND(INT(B2)=INT(C2), HOUR(B2)=HOUR(C2)), "Yes", "No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>qer-fal-092</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-21 11:09:22</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-21 17:13:45</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>8woh-k3u-23b</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>qwe-asd-99</t>
+        </is>
+      </c>
+      <c r="F3" s="2">
+        <f>IF(INT(B3)=INT(C3), "Yes", "No")</f>
+        <v/>
+      </c>
+      <c r="G3" s="2">
+        <f>IF(AND(INT(B3)=INT(C3), HOUR(B3)=HOUR(C3)), "Yes", "No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>tk-aaa-111</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-22 10:15:00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-22 18:30:00</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>wrqy-juv-978</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>cms-101</t>
+        </is>
+      </c>
+      <c r="F4" s="2">
+        <f>IF(INT(B4)=INT(C4), "Yes", "No")</f>
+        <v/>
+      </c>
+      <c r="G4" s="2">
+        <f>IF(AND(INT(B4)=INT(C4), HOUR(B4)=HOUR(C4)), "Yes", "No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>tk-bbb-222</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-23 09:10:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-23 09:45:00</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>8woh-k3u-23b</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>cms-102</t>
+        </is>
+      </c>
+      <c r="F5" s="2">
+        <f>IF(INT(B5)=INT(C5), "Yes", "No")</f>
+        <v/>
+      </c>
+      <c r="G5" s="2">
+        <f>IF(AND(INT(B5)=INT(C5), HOUR(B5)=HOUR(C5)), "Yes", "No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>tk-ccc-333</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-24 14:20:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-25 10:00:00</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>wrqy-juv-978</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>cms-103</t>
+        </is>
+      </c>
+      <c r="F6" s="2">
+        <f>IF(INT(B6)=INT(C6), "Yes", "No")</f>
+        <v/>
+      </c>
+      <c r="G6" s="2">
+        <f>IF(AND(INT(B6)=INT(C6), HOUR(B6)=HOUR(C6)), "Yes", "No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>tk-ddd-444</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-25 11:05:00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-25 11:55:00</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>wrqy-juv-978</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>cms-104</t>
+        </is>
+      </c>
+      <c r="F7" s="2">
+        <f>IF(INT(B7)=INT(C7), "Yes", "No")</f>
+        <v/>
+      </c>
+      <c r="G7" s="2">
+        <f>IF(AND(INT(B7)=INT(C7), HOUR(B7)=HOUR(C7)), "Yes", "No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>tk-eee-555</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-26 16:45:43</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-26 21:33:32</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>outlet-alpha</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>cms-105</t>
+        </is>
+      </c>
+      <c r="F8" s="2">
+        <f>IF(INT(B8)=INT(C8), "Yes", "No")</f>
+        <v/>
+      </c>
+      <c r="G8" s="2">
+        <f>IF(AND(INT(B8)=INT(C8), HOUR(B8)=HOUR(C8)), "Yes", "No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>tk-fff-666</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-27 08:30:00</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-27 08:59:00</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>outlet-alpha</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>cms-106</t>
+        </is>
+      </c>
+      <c r="F9" s="2">
+        <f>IF(INT(B9)=INT(C9), "Yes", "No")</f>
+        <v/>
+      </c>
+      <c r="G9" s="2">
+        <f>IF(AND(INT(B9)=INT(C9), HOUR(B9)=HOUR(C9)), "Yes", "No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>tk-ggg-777</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-28 12:00:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-30 12:00:00</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>8woh-k3u-23b</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>cms-107</t>
+        </is>
+      </c>
+      <c r="F10" s="2">
+        <f>IF(INT(B10)=INT(C10), "Yes", "No")</f>
+        <v/>
+      </c>
+      <c r="G10" s="2">
+        <f>IF(AND(INT(B10)=INT(C10), HOUR(B10)=HOUR(C10)), "Yes", "No")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="86" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>cms_id</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>feedback_at</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>feedback_rating</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>ticket_created_at</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>vew-iuvd-12</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2021-08-21 13:26:48</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D2">
-        <f>INDEX('ticket'!B:B, MATCH(A2, 'ticket'!E:E, 0))</f>
+      <c r="D2" s="2">
+        <f>IFERROR(INDEX(ticket!$B$2:$B$100, MATCH(A2, ticket!$E$2:$E$100, 0)), "Not Found")</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>qwe-asd-99</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>2021-08-22 09:12:34</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D3">
-        <f>INDEX('ticket'!B:B, MATCH(A3, 'ticket'!E:E, 0))</f>
+      <c r="D3" s="2">
+        <f>IFERROR(INDEX(ticket!$B$2:$B$100, MATCH(A3, ticket!$E$2:$E$100, 0)), "Not Found")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>cms-101</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-23 10:00:00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2">
+        <f>IFERROR(INDEX(ticket!$B$2:$B$100, MATCH(A4, ticket!$E$2:$E$100, 0)), "Not Found")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>cms-102</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-24 11:00:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2">
+        <f>IFERROR(INDEX(ticket!$B$2:$B$100, MATCH(A5, ticket!$E$2:$E$100, 0)), "Not Found")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>cms-104</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-26 09:00:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2">
+        <f>IFERROR(INDEX(ticket!$B$2:$B$100, MATCH(A6, ticket!$E$2:$E$100, 0)), "Not Found")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>cms-106</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2021-08-28 14:00:00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2">
+        <f>IFERROR(INDEX(ticket!$B$2:$B$100, MATCH(A7, ticket!$E$2:$E$100, 0)), "Not Found")</f>
         <v/>
       </c>
     </row>

</xml_diff>